<commit_message>
Update bank interest rate report
</commit_message>
<xml_diff>
--- a/output/interest_rate_report.xlsx
+++ b/output/interest_rate_report.xlsx
@@ -2344,12 +2344,12 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66818</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67446</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -2376,12 +2376,12 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66817</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67445</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -2408,12 +2408,12 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66816</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67444</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -2440,12 +2440,12 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66815</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67443</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -2472,12 +2472,12 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66814</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67442</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -2504,12 +2504,12 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66813</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67441</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -2536,12 +2536,12 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66812</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67440</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -2568,12 +2568,12 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66811</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67439</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -2600,12 +2600,12 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66810</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67438</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -2632,12 +2632,12 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66809</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67437</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -2664,12 +2664,12 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66808</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67435</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -2696,12 +2696,12 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66807</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67428</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -2728,12 +2728,12 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66806</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67436</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -2760,12 +2760,12 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66805</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67434</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -2792,12 +2792,12 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66803</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67432</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -2824,12 +2824,12 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66804</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67433</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -2856,12 +2856,12 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66802</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67430</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -2871,7 +2871,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Source document could not be read; all rates marked Not specified. | Ignored older duplicate: 2026-08-16 | Rastriya Banijya Bank Limited has published a notice regarding new interest rate on loan which is going to be effective from Bhadra 01, 2083</t>
+          <t>Source document could not be read; all rates marked Not specified.</t>
         </is>
       </c>
     </row>
@@ -2888,12 +2888,12 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66800</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67429</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -2920,12 +2920,12 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66799</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67427</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -2952,12 +2952,12 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66798</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67426</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -2984,12 +2984,12 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66797</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67425</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -3016,12 +3016,12 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66796</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67424</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
@@ -3048,12 +3048,12 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67049</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67423</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -3080,12 +3080,12 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66794</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67422</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -3112,12 +3112,12 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66793</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67421</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -3144,12 +3144,12 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66792</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67420</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -3176,12 +3176,12 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66791</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67419</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -3208,12 +3208,12 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66790</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67418</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
@@ -3240,12 +3240,12 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66789</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67417</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -3272,12 +3272,12 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67039</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67416</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
@@ -3304,12 +3304,12 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66787</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67415</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
@@ -3336,12 +3336,12 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66786</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67414</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
@@ -3368,12 +3368,12 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>https://merolagani.com/AnnouncementDetail.aspx?id=66785</t>
+          <t>https://merolagani.com/AnnouncementDetail.aspx?id=67413</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">

</xml_diff>